<commit_message>
Block/Item Sounds & Cleanup
</commit_message>
<xml_diff>
--- a/SoundToDo.xlsx
+++ b/SoundToDo.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hughe\AppData\Roaming\.minecraft\resourcepacks\8bit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18654B3F-0E0C-4026-828B-8B4A549733FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3DF2C5B-70CD-4127-8B8D-4193A5D463F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{0784692F-AAC4-41F3-8FDF-528C01890AB1}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="169">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="171">
   <si>
     <t>Zombie</t>
   </si>
@@ -201,18 +201,12 @@
     <t>Bucket</t>
   </si>
   <si>
-    <t>Snow</t>
-  </si>
-  <si>
     <t>Empty</t>
   </si>
   <si>
     <t>Fill</t>
   </si>
   <si>
-    <t>Lava</t>
-  </si>
-  <si>
     <t>Sand</t>
   </si>
   <si>
@@ -276,9 +270,6 @@
     <t>Climb Vine</t>
   </si>
   <si>
-    <t>Drink (&amp; Honey)</t>
-  </si>
-  <si>
     <t>Shield Block</t>
   </si>
   <si>
@@ -375,9 +366,6 @@
     <t>Item About</t>
   </si>
   <si>
-    <t>Item Spawn</t>
-  </si>
-  <si>
     <t>Ominious</t>
   </si>
   <si>
@@ -537,13 +525,31 @@
     <t>(?)</t>
   </si>
   <si>
-    <t>Knockback</t>
-  </si>
-  <si>
     <t>Bad Omen</t>
   </si>
   <si>
     <t>Trial Omen</t>
+  </si>
+  <si>
+    <t>Drink (Honey (p))</t>
+  </si>
+  <si>
+    <t>Lava (p)</t>
+  </si>
+  <si>
+    <t>Snow (v)</t>
+  </si>
+  <si>
+    <t>Knockback (v)</t>
+  </si>
+  <si>
+    <t>Bat</t>
+  </si>
+  <si>
+    <t>Enderman</t>
+  </si>
+  <si>
+    <t>Item Spawn (p)</t>
   </si>
 </sst>
 </file>
@@ -606,13 +612,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -947,13 +952,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{860EC8D9-E5E7-4F7C-95C9-48163BD097DB}">
-  <dimension ref="A1:M19"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="11" max="11" width="13.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B1" t="s">
         <v>0</v>
       </c>
@@ -976,7 +981,7 @@
         <v>48</v>
       </c>
       <c r="I1" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="K1" t="s">
         <v>47</v>
@@ -984,8 +989,14 @@
       <c r="M1" t="s">
         <v>49</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="O1" t="s">
+        <v>168</v>
+      </c>
+      <c r="P1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -1000,13 +1011,13 @@
         <v>8</v>
       </c>
       <c r="J2" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="L2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -1020,16 +1031,16 @@
         <v>8</v>
       </c>
       <c r="J3" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="L3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="M3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -1043,13 +1054,13 @@
         <v>8</v>
       </c>
       <c r="J4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="L4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -1066,15 +1077,15 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
       <c r="H6" s="3" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="L6" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B7" t="s">
         <v>18</v>
       </c>
@@ -1088,10 +1099,10 @@
         <v>15</v>
       </c>
       <c r="L7" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -1100,10 +1111,10 @@
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="L8" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -1112,52 +1123,52 @@
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="L9" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>35</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>34</v>
       </c>
       <c r="L10" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B11" s="1" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>32</v>
       </c>
       <c r="L11" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>39</v>
@@ -1166,12 +1177,12 @@
         <v>23</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>46</v>
@@ -1180,15 +1191,15 @@
         <v>40</v>
       </c>
       <c r="L13" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
         <v>50</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>45</v>
@@ -1197,41 +1208,41 @@
         <v>52</v>
       </c>
       <c r="L14" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B15" s="1" t="s">
         <v>51</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
-        <v>139</v>
+        <v>135</v>
       </c>
       <c r="C16" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B18" s="1" t="s">
-        <v>135</v>
+        <v>131</v>
       </c>
     </row>
     <row r="19" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B19" s="1" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -1258,22 +1269,23 @@
         <v>22</v>
       </c>
       <c r="K1" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="L1" t="s">
         <v>36</v>
       </c>
       <c r="O1" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="R1" t="s">
-        <v>155</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>142</v>
-      </c>
+        <v>138</v>
+      </c>
+      <c r="B2" s="1"/>
       <c r="D2" t="s">
         <v>26</v>
       </c>
@@ -1286,11 +1298,13 @@
         <v>20</v>
       </c>
       <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
       <c r="N2" s="2" t="s">
-        <v>158</v>
-      </c>
+        <v>154</v>
+      </c>
+      <c r="O2" s="1"/>
       <c r="Q2" t="s">
-        <v>160</v>
+        <v>156</v>
       </c>
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.3">
@@ -1310,8 +1324,9 @@
         <v>21</v>
       </c>
       <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
       <c r="N3" s="2" t="s">
-        <v>159</v>
+        <v>155</v>
       </c>
       <c r="O3" s="1"/>
       <c r="Q3" t="s">
@@ -1321,7 +1336,7 @@
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B4" s="1"/>
       <c r="D4" t="s">
@@ -1333,10 +1348,10 @@
       </c>
       <c r="H4" s="1"/>
       <c r="K4" s="1" t="s">
-        <v>145</v>
-      </c>
-      <c r="L4" t="s">
-        <v>150</v>
+        <v>141</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>146</v>
       </c>
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.3">
@@ -1350,16 +1365,16 @@
     </row>
     <row r="6" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B6" s="1"/>
       <c r="Q6" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
     </row>
     <row r="7" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B7" s="1"/>
       <c r="E7" t="s">
@@ -1372,17 +1387,18 @@
         <v>53</v>
       </c>
       <c r="N7" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="P7" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="Q7" s="1"/>
     </row>
     <row r="8" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>76</v>
-      </c>
+        <v>74</v>
+      </c>
+      <c r="B8" s="1"/>
       <c r="D8" t="s">
         <v>7</v>
       </c>
@@ -1392,34 +1408,37 @@
       </c>
       <c r="H8" s="1"/>
       <c r="J8" t="s">
-        <v>55</v>
-      </c>
+        <v>54</v>
+      </c>
+      <c r="K8" s="1"/>
       <c r="M8" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="N8" s="1"/>
       <c r="P8" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="Q8" s="1"/>
     </row>
     <row r="9" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>79</v>
-      </c>
+        <v>164</v>
+      </c>
+      <c r="B9" s="1"/>
       <c r="D9" s="2" t="s">
         <v>37</v>
       </c>
       <c r="E9" s="1"/>
       <c r="G9" s="2" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
       <c r="H9" s="1"/>
       <c r="J9" t="s">
-        <v>56</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="K9" s="1"/>
       <c r="M9" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="N9" s="1"/>
       <c r="P9" t="s">
@@ -1429,7 +1448,7 @@
     </row>
     <row r="10" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="B10" s="1"/>
       <c r="D10" s="2" t="s">
@@ -1437,184 +1456,194 @@
       </c>
       <c r="E10" s="1"/>
       <c r="J10" s="2"/>
-      <c r="K10" s="5" t="s">
-        <v>54</v>
+      <c r="K10" s="1" t="s">
+        <v>166</v>
       </c>
       <c r="M10" s="2"/>
       <c r="N10" s="1" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
     </row>
     <row r="11" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="B11" s="1"/>
       <c r="J11" s="2"/>
-      <c r="K11" s="5" t="s">
-        <v>57</v>
+      <c r="K11" s="1" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="12" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>81</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="B12" s="1"/>
       <c r="J12" s="2"/>
-      <c r="K12" s="5" t="s">
-        <v>152</v>
+      <c r="K12" s="1" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="13" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>95</v>
-      </c>
+        <v>92</v>
+      </c>
+      <c r="B13" s="1"/>
     </row>
     <row r="14" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B14" s="1"/>
       <c r="E14" t="s">
         <v>12</v>
       </c>
       <c r="I14" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="L14" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="O14" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="R14" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
     </row>
     <row r="15" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>84</v>
-      </c>
+        <v>81</v>
+      </c>
+      <c r="B15" s="1"/>
       <c r="D15" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="E15" s="1"/>
       <c r="H15" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="K15" t="s">
-        <v>90</v>
-      </c>
+        <v>87</v>
+      </c>
+      <c r="L15" s="1"/>
       <c r="N15" t="s">
         <v>7</v>
       </c>
+      <c r="O15" s="1"/>
       <c r="Q15" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="16" spans="1:18" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B16" s="1"/>
       <c r="D16" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="E16" s="1"/>
       <c r="H16" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="K16" t="s">
-        <v>91</v>
-      </c>
+        <v>88</v>
+      </c>
+      <c r="L16" s="1"/>
       <c r="N16" t="s">
-        <v>106</v>
-      </c>
+        <v>103</v>
+      </c>
+      <c r="O16" s="1"/>
       <c r="Q16" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
     </row>
     <row r="17" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>154</v>
-      </c>
+        <v>150</v>
+      </c>
+      <c r="B17" s="1"/>
       <c r="D17" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="E17" s="1"/>
       <c r="H17" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="K17" s="2"/>
-      <c r="L17" s="5" t="s">
-        <v>153</v>
+      <c r="L17" s="1" t="s">
+        <v>149</v>
       </c>
       <c r="N17" t="s">
-        <v>149</v>
-      </c>
+        <v>145</v>
+      </c>
+      <c r="O17" s="1"/>
       <c r="Q17" t="s">
-        <v>133</v>
+        <v>129</v>
       </c>
     </row>
     <row r="18" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B18" s="1"/>
       <c r="D18" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="E18" s="1"/>
       <c r="H18" t="s">
         <v>7</v>
       </c>
       <c r="K18" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="L18" s="1"/>
       <c r="N18" t="s">
-        <v>109</v>
-      </c>
+        <v>106</v>
+      </c>
+      <c r="O18" s="1"/>
       <c r="Q18" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
     </row>
     <row r="19" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B19" s="1"/>
       <c r="D19" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="E19" s="1"/>
       <c r="H19" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="K19" t="s">
         <v>23</v>
       </c>
       <c r="L19" s="1"/>
-      <c r="N19" t="s">
-        <v>20</v>
-      </c>
-      <c r="O19" s="1"/>
+      <c r="O19" s="1" t="s">
+        <v>170</v>
+      </c>
       <c r="Q19" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="20" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>101</v>
-      </c>
+        <v>98</v>
+      </c>
+      <c r="B20" s="1"/>
       <c r="D20" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="E20" s="1"/>
       <c r="H20" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="N20" t="s">
-        <v>107</v>
+        <v>20</v>
       </c>
       <c r="O20" s="1"/>
       <c r="Q20" t="s">
@@ -1623,20 +1652,21 @@
     </row>
     <row r="21" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>102</v>
-      </c>
+        <v>99</v>
+      </c>
+      <c r="B21" s="1"/>
       <c r="D21" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="E21" s="1"/>
       <c r="F21" t="s">
-        <v>161</v>
+        <v>157</v>
       </c>
       <c r="H21" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="N21" t="s">
-        <v>21</v>
+        <v>104</v>
       </c>
       <c r="O21" s="1"/>
       <c r="Q21" t="s">
@@ -1645,72 +1675,77 @@
     </row>
     <row r="22" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="B22" s="1"/>
       <c r="D22" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="E22" s="1"/>
       <c r="F22" t="s">
-        <v>162</v>
+        <v>158</v>
       </c>
       <c r="N22" t="s">
-        <v>113</v>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="O22" s="1"/>
       <c r="Q22" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
     </row>
     <row r="23" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="D23" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="E23" s="1"/>
       <c r="F23" t="s">
-        <v>164</v>
+        <v>160</v>
       </c>
       <c r="N23" t="s">
-        <v>110</v>
-      </c>
+        <v>109</v>
+      </c>
+      <c r="O23" s="1"/>
     </row>
     <row r="24" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="D24" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E24" s="1"/>
       <c r="F24" t="s">
-        <v>163</v>
+        <v>159</v>
       </c>
       <c r="N24" t="s">
-        <v>111</v>
-      </c>
+        <v>107</v>
+      </c>
+      <c r="O24" s="1"/>
     </row>
     <row r="25" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="D25" s="2"/>
       <c r="E25" s="1" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="F25" t="s">
-        <v>165</v>
+        <v>161</v>
       </c>
       <c r="N25" t="s">
-        <v>112</v>
-      </c>
+        <v>108</v>
+      </c>
+      <c r="O25" s="1"/>
     </row>
     <row r="26" spans="1:17" x14ac:dyDescent="0.3">
       <c r="D26" t="s">
-        <v>119</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="E26" s="1"/>
     </row>
     <row r="27" spans="1:17" x14ac:dyDescent="0.3">
       <c r="D27" t="s">

</xml_diff>

<commit_message>
Spider/Silverfish/Chicken Sounds + GUI
</commit_message>
<xml_diff>
--- a/SoundToDo.xlsx
+++ b/SoundToDo.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\hughe\AppData\Roaming\.minecraft\resourcepacks\8bit\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{974482C2-A379-4CE5-B4D9-59451ABA7B2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6C24A43-90B1-4CBA-ADA8-4F36E0C9F727}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{0784692F-AAC4-41F3-8FDF-528C01890AB1}"/>
+    <workbookView xWindow="-19310" yWindow="-110" windowWidth="19420" windowHeight="11020" xr2:uid="{0784692F-AAC4-41F3-8FDF-528C01890AB1}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -1066,12 +1066,16 @@
       <c r="C2" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E2" t="s">
+      <c r="D2" s="1"/>
+      <c r="E2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="G2" s="1"/>
+      <c r="H2" s="1"/>
+      <c r="I2" s="1"/>
       <c r="J2" t="s">
         <v>62</v>
       </c>
@@ -1091,15 +1095,18 @@
       <c r="C3" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E3" t="s">
+      <c r="D3" s="1"/>
+      <c r="E3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="1" t="s">
         <v>8</v>
       </c>
       <c r="G3" s="7" t="s">
         <v>173</v>
       </c>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
       <c r="J3" t="s">
         <v>63</v>
       </c>
@@ -1117,12 +1124,15 @@
       <c r="C4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E4" t="s">
+      <c r="D4" s="1"/>
+      <c r="E4" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="G4" s="1"/>
+      <c r="H4" s="1"/>
       <c r="I4" s="7" t="s">
         <v>173</v>
       </c>
@@ -1143,12 +1153,16 @@
       <c r="C5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E5" t="s">
+      <c r="D5" s="1"/>
+      <c r="E5" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="1" t="s">
         <v>8</v>
       </c>
+      <c r="G5" s="1"/>
+      <c r="H5" s="1"/>
+      <c r="I5" s="1"/>
       <c r="L5" t="s">
         <v>65</v>
       </c>

</xml_diff>